<commit_message>
Implemented time environment into example files
</commit_message>
<xml_diff>
--- a/examples/hardware/sdynpy_system.xlsx
+++ b/examples/hardware/sdynpy_system.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W32"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,7 +566,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1004X+</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1053,7 +1053,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -1061,11 +1061,7 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
@@ -1076,7 +1072,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1086,7 +1082,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1004Y+</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1104,7 +1100,7 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -1112,11 +1108,7 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
@@ -1127,7 +1119,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1137,7 +1129,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1004Z+</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1155,7 +1147,7 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1163,11 +1155,7 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
@@ -1178,7 +1166,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1188,7 +1176,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1004X+</t>
+          <t>1020X+</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1225,7 +1213,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1235,7 +1223,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1004Y+</t>
+          <t>1020Y+</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1272,7 +1260,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1282,7 +1270,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1004Z+</t>
+          <t>1020Z+</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1319,7 +1307,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1329,7 +1317,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1012X+</t>
+          <t>1065X+</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1366,7 +1354,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1376,7 +1364,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1012Y+</t>
+          <t>1065Y+</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1413,7 +1401,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1423,7 +1411,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1012Z+</t>
+          <t>1065Z+</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1460,7 +1448,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>1049</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1470,7 +1458,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1020X+</t>
+          <t>1049X+</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1507,7 +1495,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>1049</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1517,7 +1505,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1020Y+</t>
+          <t>1049Y+</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1554,7 +1542,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>1049</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1564,7 +1552,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1020Z+</t>
+          <t>1049Z+</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1594,429 +1582,6 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1065</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>X+</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>1065X+</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1065</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Y+</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>1065Y+</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1065</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Z+</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>1065Z+</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1057</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>X+</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>1057X+</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>1057</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Y+</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>1057Y+</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1057</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Z+</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>1057Z+</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>1049</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>X+</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>1049X+</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>1049</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Y+</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>1049Y+</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>1049</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Z+</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>1049Z+</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Acceleration</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Got state space system working with new architecture
</commit_message>
<xml_diff>
--- a/examples/hardware/sdynpy_system.xlsx
+++ b/examples/hardware/sdynpy_system.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1004X+</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -594,7 +594,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -602,11 +602,7 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
@@ -617,7 +613,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -627,7 +623,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1004Y+</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -645,7 +641,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
@@ -653,11 +649,7 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
@@ -668,7 +660,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -678,7 +670,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1004Z+</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -696,7 +688,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -704,11 +696,7 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
@@ -719,7 +707,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -729,7 +717,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1020X+</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -747,7 +735,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -755,11 +743,7 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
@@ -770,7 +754,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -780,7 +764,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1020Y+</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -798,7 +782,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -806,11 +790,7 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
@@ -821,7 +801,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -831,7 +811,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1020Z+</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -849,7 +829,7 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -857,11 +837,7 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
@@ -872,7 +848,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -882,7 +858,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1065X+</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -900,7 +876,7 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -908,11 +884,7 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
@@ -923,7 +895,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -933,7 +905,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1065Y+</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -951,7 +923,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -959,11 +931,7 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
@@ -974,7 +942,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -984,7 +952,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>1065Z+</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -1002,7 +970,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Acceleration</t>
         </is>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -1010,11 +978,7 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
@@ -1025,7 +989,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1049</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1035,7 +999,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1004X+</t>
+          <t>1049X+</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1072,7 +1036,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1049</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1082,7 +1046,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1004Y+</t>
+          <t>1049Y+</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1119,7 +1083,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>1049</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1129,7 +1093,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1004Z+</t>
+          <t>1049Z+</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1166,7 +1130,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1176,7 +1140,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1020X+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1194,7 +1158,7 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -1202,7 +1166,11 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
@@ -1213,7 +1181,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1223,7 +1191,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1020Y+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1241,7 +1209,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -1249,7 +1217,11 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
@@ -1260,7 +1232,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1270,7 +1242,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1020Z+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1288,7 +1260,7 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
@@ -1296,7 +1268,11 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
@@ -1307,7 +1283,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1065</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1317,7 +1293,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1065X+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1335,7 +1311,7 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -1343,7 +1319,11 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
@@ -1354,7 +1334,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1065</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1364,7 +1344,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1065Y+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1382,7 +1362,7 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -1390,7 +1370,11 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
@@ -1401,7 +1385,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1065</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1411,7 +1395,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1065Z+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1429,7 +1413,7 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O20" t="inlineStr"/>
@@ -1437,7 +1421,11 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
@@ -1448,7 +1436,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1049</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1458,7 +1446,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1049X+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -1476,7 +1464,7 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
@@ -1484,7 +1472,11 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
@@ -1495,7 +1487,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1049</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1505,7 +1497,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1049Y+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1523,7 +1515,7 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
@@ -1531,7 +1523,11 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
@@ -1542,7 +1538,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1049</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1552,7 +1548,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1049Z+</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1570,7 +1566,7 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="O23" t="inlineStr"/>
@@ -1578,7 +1574,11 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>

</xml_diff>